<commit_message>
txt y csv ej 2
</commit_message>
<xml_diff>
--- a/src/main/resources/empleados.xlsx
+++ b/src/main/resources/empleados.xlsx
@@ -312,40 +312,40 @@
         <v>16</v>
       </c>
       <c r="D2" t="n" s="0">
-        <v>1724.46</v>
+        <v>1797.83</v>
       </c>
       <c r="E2" t="n" s="0">
-        <v>1768.99</v>
+        <v>1877.89</v>
       </c>
       <c r="F2" t="n" s="0">
-        <v>1490.35</v>
+        <v>1617.91</v>
       </c>
       <c r="G2" t="n" s="0">
-        <v>1734.64</v>
+        <v>1953.09</v>
       </c>
       <c r="H2" t="n" s="0">
-        <v>1442.25</v>
+        <v>1522.75</v>
       </c>
       <c r="I2" t="n" s="0">
-        <v>1742.02</v>
+        <v>1307.89</v>
       </c>
       <c r="J2" t="n" s="0">
-        <v>1867.61</v>
+        <v>1325.82</v>
       </c>
       <c r="K2" t="n" s="0">
-        <v>1202.65</v>
+        <v>1331.02</v>
       </c>
       <c r="L2" t="n" s="0">
-        <v>1906.47</v>
+        <v>1635.55</v>
       </c>
       <c r="M2" t="n" s="0">
-        <v>1483.59</v>
+        <v>1578.33</v>
       </c>
       <c r="N2" t="n" s="0">
-        <v>1321.54</v>
+        <v>1945.21</v>
       </c>
       <c r="O2" t="n" s="0">
-        <v>1656.86</v>
+        <v>1965.47</v>
       </c>
     </row>
     <row r="3">
@@ -359,40 +359,40 @@
         <v>18</v>
       </c>
       <c r="D3" t="n" s="0">
-        <v>1636.64</v>
+        <v>1201.41</v>
       </c>
       <c r="E3" t="n" s="0">
-        <v>1998.29</v>
+        <v>1681.94</v>
       </c>
       <c r="F3" t="n" s="0">
-        <v>1518.43</v>
+        <v>1492.86</v>
       </c>
       <c r="G3" t="n" s="0">
-        <v>1677.01</v>
+        <v>1244.81</v>
       </c>
       <c r="H3" t="n" s="0">
-        <v>1237.79</v>
+        <v>1729.26</v>
       </c>
       <c r="I3" t="n" s="0">
-        <v>1595.39</v>
+        <v>1223.11</v>
       </c>
       <c r="J3" t="n" s="0">
-        <v>1459.32</v>
+        <v>1558.23</v>
       </c>
       <c r="K3" t="n" s="0">
-        <v>1238.25</v>
+        <v>1793.46</v>
       </c>
       <c r="L3" t="n" s="0">
-        <v>1257.44</v>
+        <v>1856.72</v>
       </c>
       <c r="M3" t="n" s="0">
-        <v>1238.5</v>
+        <v>1977.12</v>
       </c>
       <c r="N3" t="n" s="0">
-        <v>1946.76</v>
+        <v>1310.34</v>
       </c>
       <c r="O3" t="n" s="0">
-        <v>1246.66</v>
+        <v>1216.14</v>
       </c>
     </row>
     <row r="4">
@@ -406,40 +406,40 @@
         <v>20</v>
       </c>
       <c r="D4" t="n" s="0">
-        <v>1256.28</v>
+        <v>1846.42</v>
       </c>
       <c r="E4" t="n" s="0">
-        <v>1998.11</v>
+        <v>1440.97</v>
       </c>
       <c r="F4" t="n" s="0">
-        <v>1996.59</v>
+        <v>1615.8</v>
       </c>
       <c r="G4" t="n" s="0">
-        <v>1711.69</v>
+        <v>1645.61</v>
       </c>
       <c r="H4" t="n" s="0">
-        <v>1505.57</v>
+        <v>1237.15</v>
       </c>
       <c r="I4" t="n" s="0">
-        <v>1345.59</v>
+        <v>1813.88</v>
       </c>
       <c r="J4" t="n" s="0">
-        <v>1261.67</v>
+        <v>1552.62</v>
       </c>
       <c r="K4" t="n" s="0">
-        <v>1313.75</v>
+        <v>1938.82</v>
       </c>
       <c r="L4" t="n" s="0">
-        <v>1987.87</v>
+        <v>1831.86</v>
       </c>
       <c r="M4" t="n" s="0">
-        <v>1672.79</v>
+        <v>1465.47</v>
       </c>
       <c r="N4" t="n" s="0">
-        <v>1409.67</v>
+        <v>1255.13</v>
       </c>
       <c r="O4" t="n" s="0">
-        <v>1882.24</v>
+        <v>1498.56</v>
       </c>
     </row>
     <row r="5">
@@ -453,40 +453,40 @@
         <v>22</v>
       </c>
       <c r="D5" t="n" s="0">
-        <v>1265.53</v>
+        <v>1267.5</v>
       </c>
       <c r="E5" t="n" s="0">
-        <v>1889.94</v>
+        <v>1593.95</v>
       </c>
       <c r="F5" t="n" s="0">
-        <v>1298.29</v>
+        <v>1301.13</v>
       </c>
       <c r="G5" t="n" s="0">
-        <v>1281.25</v>
+        <v>1254.53</v>
       </c>
       <c r="H5" t="n" s="0">
-        <v>1895.09</v>
+        <v>1300.25</v>
       </c>
       <c r="I5" t="n" s="0">
-        <v>1649.88</v>
+        <v>1246.18</v>
       </c>
       <c r="J5" t="n" s="0">
-        <v>1716.8</v>
+        <v>1753.27</v>
       </c>
       <c r="K5" t="n" s="0">
-        <v>1407.36</v>
+        <v>1519.84</v>
       </c>
       <c r="L5" t="n" s="0">
-        <v>1403.66</v>
+        <v>1252.75</v>
       </c>
       <c r="M5" t="n" s="0">
-        <v>1265.54</v>
+        <v>1966.09</v>
       </c>
       <c r="N5" t="n" s="0">
-        <v>1813.75</v>
+        <v>1492.41</v>
       </c>
       <c r="O5" t="n" s="0">
-        <v>1235.75</v>
+        <v>1846.18</v>
       </c>
     </row>
     <row r="6">
@@ -500,40 +500,40 @@
         <v>24</v>
       </c>
       <c r="D6" t="n" s="0">
-        <v>1206.96</v>
+        <v>1608.35</v>
       </c>
       <c r="E6" t="n" s="0">
-        <v>1532.69</v>
+        <v>1457.33</v>
       </c>
       <c r="F6" t="n" s="0">
-        <v>1906.16</v>
+        <v>1431.36</v>
       </c>
       <c r="G6" t="n" s="0">
-        <v>1708.12</v>
+        <v>1432.51</v>
       </c>
       <c r="H6" t="n" s="0">
-        <v>1836.68</v>
+        <v>1500.7</v>
       </c>
       <c r="I6" t="n" s="0">
-        <v>1239.0</v>
+        <v>1390.77</v>
       </c>
       <c r="J6" t="n" s="0">
-        <v>1366.85</v>
+        <v>1973.36</v>
       </c>
       <c r="K6" t="n" s="0">
-        <v>1337.79</v>
+        <v>1699.66</v>
       </c>
       <c r="L6" t="n" s="0">
-        <v>1858.3</v>
+        <v>1635.09</v>
       </c>
       <c r="M6" t="n" s="0">
-        <v>1735.36</v>
+        <v>1456.8</v>
       </c>
       <c r="N6" t="n" s="0">
-        <v>1311.6</v>
+        <v>1280.28</v>
       </c>
       <c r="O6" t="n" s="0">
-        <v>1514.39</v>
+        <v>1324.81</v>
       </c>
     </row>
     <row r="7">
@@ -547,40 +547,40 @@
         <v>26</v>
       </c>
       <c r="D7" t="n" s="0">
-        <v>1498.76</v>
+        <v>1791.56</v>
       </c>
       <c r="E7" t="n" s="0">
-        <v>1564.75</v>
+        <v>1556.89</v>
       </c>
       <c r="F7" t="n" s="0">
-        <v>1859.43</v>
+        <v>1741.58</v>
       </c>
       <c r="G7" t="n" s="0">
-        <v>1422.73</v>
+        <v>1937.14</v>
       </c>
       <c r="H7" t="n" s="0">
-        <v>1466.55</v>
+        <v>1497.67</v>
       </c>
       <c r="I7" t="n" s="0">
-        <v>1388.48</v>
+        <v>1848.77</v>
       </c>
       <c r="J7" t="n" s="0">
-        <v>1214.23</v>
+        <v>1485.34</v>
       </c>
       <c r="K7" t="n" s="0">
-        <v>1847.19</v>
+        <v>1807.88</v>
       </c>
       <c r="L7" t="n" s="0">
-        <v>1935.21</v>
+        <v>1722.56</v>
       </c>
       <c r="M7" t="n" s="0">
-        <v>1919.33</v>
+        <v>1803.52</v>
       </c>
       <c r="N7" t="n" s="0">
-        <v>1917.64</v>
+        <v>1849.11</v>
       </c>
       <c r="O7" t="n" s="0">
-        <v>1315.35</v>
+        <v>1224.99</v>
       </c>
     </row>
     <row r="8">
@@ -594,40 +594,40 @@
         <v>28</v>
       </c>
       <c r="D8" t="n" s="0">
-        <v>1374.35</v>
+        <v>1331.74</v>
       </c>
       <c r="E8" t="n" s="0">
-        <v>1265.37</v>
+        <v>1702.98</v>
       </c>
       <c r="F8" t="n" s="0">
-        <v>1947.93</v>
+        <v>1228.49</v>
       </c>
       <c r="G8" t="n" s="0">
-        <v>1841.33</v>
+        <v>1624.74</v>
       </c>
       <c r="H8" t="n" s="0">
-        <v>1850.86</v>
+        <v>1355.77</v>
       </c>
       <c r="I8" t="n" s="0">
-        <v>1408.04</v>
+        <v>1499.99</v>
       </c>
       <c r="J8" t="n" s="0">
-        <v>1291.27</v>
+        <v>1847.6</v>
       </c>
       <c r="K8" t="n" s="0">
-        <v>1761.36</v>
+        <v>1359.56</v>
       </c>
       <c r="L8" t="n" s="0">
-        <v>1785.8</v>
+        <v>1663.86</v>
       </c>
       <c r="M8" t="n" s="0">
-        <v>1282.37</v>
+        <v>1483.81</v>
       </c>
       <c r="N8" t="n" s="0">
-        <v>1786.94</v>
+        <v>1546.04</v>
       </c>
       <c r="O8" t="n" s="0">
-        <v>1411.5</v>
+        <v>1413.53</v>
       </c>
     </row>
     <row r="9">
@@ -641,40 +641,40 @@
         <v>30</v>
       </c>
       <c r="D9" t="n" s="0">
-        <v>1341.34</v>
+        <v>1597.15</v>
       </c>
       <c r="E9" t="n" s="0">
-        <v>1297.02</v>
+        <v>1537.32</v>
       </c>
       <c r="F9" t="n" s="0">
-        <v>1849.14</v>
+        <v>1653.05</v>
       </c>
       <c r="G9" t="n" s="0">
-        <v>1278.77</v>
+        <v>1633.76</v>
       </c>
       <c r="H9" t="n" s="0">
-        <v>1224.76</v>
+        <v>1704.24</v>
       </c>
       <c r="I9" t="n" s="0">
-        <v>1526.02</v>
+        <v>1342.38</v>
       </c>
       <c r="J9" t="n" s="0">
-        <v>1693.71</v>
+        <v>1619.98</v>
       </c>
       <c r="K9" t="n" s="0">
-        <v>1364.81</v>
+        <v>1728.3</v>
       </c>
       <c r="L9" t="n" s="0">
-        <v>1935.36</v>
+        <v>1535.13</v>
       </c>
       <c r="M9" t="n" s="0">
-        <v>1623.92</v>
+        <v>1884.14</v>
       </c>
       <c r="N9" t="n" s="0">
-        <v>1348.87</v>
+        <v>1708.31</v>
       </c>
       <c r="O9" t="n" s="0">
-        <v>1232.44</v>
+        <v>1387.78</v>
       </c>
     </row>
     <row r="10">
@@ -688,40 +688,40 @@
         <v>32</v>
       </c>
       <c r="D10" t="n" s="0">
-        <v>1743.09</v>
+        <v>1688.07</v>
       </c>
       <c r="E10" t="n" s="0">
-        <v>1560.42</v>
+        <v>1424.6</v>
       </c>
       <c r="F10" t="n" s="0">
-        <v>1805.0</v>
+        <v>1481.07</v>
       </c>
       <c r="G10" t="n" s="0">
-        <v>1363.09</v>
+        <v>1220.41</v>
       </c>
       <c r="H10" t="n" s="0">
-        <v>1576.01</v>
+        <v>1366.64</v>
       </c>
       <c r="I10" t="n" s="0">
-        <v>1740.17</v>
+        <v>1960.27</v>
       </c>
       <c r="J10" t="n" s="0">
-        <v>1958.94</v>
+        <v>1721.29</v>
       </c>
       <c r="K10" t="n" s="0">
-        <v>1234.83</v>
+        <v>1546.88</v>
       </c>
       <c r="L10" t="n" s="0">
-        <v>1507.17</v>
+        <v>1993.39</v>
       </c>
       <c r="M10" t="n" s="0">
-        <v>1767.83</v>
+        <v>1448.48</v>
       </c>
       <c r="N10" t="n" s="0">
-        <v>1334.51</v>
+        <v>1901.89</v>
       </c>
       <c r="O10" t="n" s="0">
-        <v>1937.84</v>
+        <v>1883.53</v>
       </c>
     </row>
     <row r="11">
@@ -735,40 +735,40 @@
         <v>34</v>
       </c>
       <c r="D11" t="n" s="0">
-        <v>1469.46</v>
+        <v>1338.85</v>
       </c>
       <c r="E11" t="n" s="0">
-        <v>1438.21</v>
+        <v>1981.01</v>
       </c>
       <c r="F11" t="n" s="0">
-        <v>1311.31</v>
+        <v>1657.29</v>
       </c>
       <c r="G11" t="n" s="0">
-        <v>1576.08</v>
+        <v>1749.54</v>
       </c>
       <c r="H11" t="n" s="0">
-        <v>1390.66</v>
+        <v>1563.71</v>
       </c>
       <c r="I11" t="n" s="0">
-        <v>1875.66</v>
+        <v>1803.77</v>
       </c>
       <c r="J11" t="n" s="0">
-        <v>1770.0</v>
+        <v>1257.79</v>
       </c>
       <c r="K11" t="n" s="0">
-        <v>1761.23</v>
+        <v>1265.63</v>
       </c>
       <c r="L11" t="n" s="0">
-        <v>1928.82</v>
+        <v>1734.73</v>
       </c>
       <c r="M11" t="n" s="0">
-        <v>1916.52</v>
+        <v>1225.33</v>
       </c>
       <c r="N11" t="n" s="0">
-        <v>1262.71</v>
+        <v>1663.27</v>
       </c>
       <c r="O11" t="n" s="0">
-        <v>1586.59</v>
+        <v>1868.97</v>
       </c>
     </row>
     <row r="12">
@@ -782,40 +782,40 @@
         <v>36</v>
       </c>
       <c r="D12" t="n" s="0">
-        <v>1201.65</v>
+        <v>1563.52</v>
       </c>
       <c r="E12" t="n" s="0">
-        <v>1622.92</v>
+        <v>1426.97</v>
       </c>
       <c r="F12" t="n" s="0">
-        <v>1443.26</v>
+        <v>1334.11</v>
       </c>
       <c r="G12" t="n" s="0">
-        <v>1576.07</v>
+        <v>1350.88</v>
       </c>
       <c r="H12" t="n" s="0">
-        <v>1341.68</v>
+        <v>1930.51</v>
       </c>
       <c r="I12" t="n" s="0">
-        <v>1235.79</v>
+        <v>1381.11</v>
       </c>
       <c r="J12" t="n" s="0">
-        <v>1742.63</v>
+        <v>1802.37</v>
       </c>
       <c r="K12" t="n" s="0">
-        <v>1435.16</v>
+        <v>1731.15</v>
       </c>
       <c r="L12" t="n" s="0">
-        <v>1372.46</v>
+        <v>1994.73</v>
       </c>
       <c r="M12" t="n" s="0">
-        <v>1519.38</v>
+        <v>1504.97</v>
       </c>
       <c r="N12" t="n" s="0">
-        <v>1750.71</v>
+        <v>1457.58</v>
       </c>
       <c r="O12" t="n" s="0">
-        <v>1587.88</v>
+        <v>1614.59</v>
       </c>
     </row>
     <row r="13">
@@ -829,40 +829,40 @@
         <v>38</v>
       </c>
       <c r="D13" t="n" s="0">
-        <v>1389.11</v>
+        <v>1553.2</v>
       </c>
       <c r="E13" t="n" s="0">
-        <v>1519.29</v>
+        <v>1720.37</v>
       </c>
       <c r="F13" t="n" s="0">
-        <v>1666.3</v>
+        <v>1876.84</v>
       </c>
       <c r="G13" t="n" s="0">
-        <v>1465.85</v>
+        <v>1832.57</v>
       </c>
       <c r="H13" t="n" s="0">
-        <v>1340.01</v>
+        <v>1602.28</v>
       </c>
       <c r="I13" t="n" s="0">
-        <v>1850.37</v>
+        <v>1860.35</v>
       </c>
       <c r="J13" t="n" s="0">
-        <v>1503.16</v>
+        <v>1330.14</v>
       </c>
       <c r="K13" t="n" s="0">
-        <v>1722.37</v>
+        <v>1554.47</v>
       </c>
       <c r="L13" t="n" s="0">
-        <v>1844.5</v>
+        <v>1366.26</v>
       </c>
       <c r="M13" t="n" s="0">
-        <v>1350.48</v>
+        <v>1857.92</v>
       </c>
       <c r="N13" t="n" s="0">
-        <v>1890.54</v>
+        <v>1817.25</v>
       </c>
       <c r="O13" t="n" s="0">
-        <v>1376.77</v>
+        <v>1660.69</v>
       </c>
     </row>
     <row r="14">
@@ -876,40 +876,40 @@
         <v>40</v>
       </c>
       <c r="D14" t="n" s="0">
-        <v>1245.05</v>
+        <v>1996.98</v>
       </c>
       <c r="E14" t="n" s="0">
-        <v>1480.56</v>
+        <v>1871.47</v>
       </c>
       <c r="F14" t="n" s="0">
-        <v>1682.49</v>
+        <v>1943.3</v>
       </c>
       <c r="G14" t="n" s="0">
-        <v>1551.18</v>
+        <v>1401.18</v>
       </c>
       <c r="H14" t="n" s="0">
-        <v>1280.19</v>
+        <v>1711.59</v>
       </c>
       <c r="I14" t="n" s="0">
-        <v>1421.12</v>
+        <v>1646.27</v>
       </c>
       <c r="J14" t="n" s="0">
-        <v>1390.96</v>
+        <v>1716.47</v>
       </c>
       <c r="K14" t="n" s="0">
-        <v>1743.7</v>
+        <v>1220.38</v>
       </c>
       <c r="L14" t="n" s="0">
-        <v>1778.29</v>
+        <v>1923.63</v>
       </c>
       <c r="M14" t="n" s="0">
-        <v>1409.65</v>
+        <v>1980.59</v>
       </c>
       <c r="N14" t="n" s="0">
-        <v>1483.65</v>
+        <v>1351.08</v>
       </c>
       <c r="O14" t="n" s="0">
-        <v>1689.34</v>
+        <v>1911.36</v>
       </c>
     </row>
     <row r="15">
@@ -923,40 +923,40 @@
         <v>42</v>
       </c>
       <c r="D15" t="n" s="0">
-        <v>1810.12</v>
+        <v>1335.98</v>
       </c>
       <c r="E15" t="n" s="0">
-        <v>1282.98</v>
+        <v>1560.08</v>
       </c>
       <c r="F15" t="n" s="0">
-        <v>1238.18</v>
+        <v>1586.22</v>
       </c>
       <c r="G15" t="n" s="0">
-        <v>1791.92</v>
+        <v>1969.34</v>
       </c>
       <c r="H15" t="n" s="0">
-        <v>1201.62</v>
+        <v>1402.75</v>
       </c>
       <c r="I15" t="n" s="0">
-        <v>1433.32</v>
+        <v>1242.91</v>
       </c>
       <c r="J15" t="n" s="0">
-        <v>1919.9</v>
+        <v>1479.8</v>
       </c>
       <c r="K15" t="n" s="0">
-        <v>1467.15</v>
+        <v>1946.25</v>
       </c>
       <c r="L15" t="n" s="0">
-        <v>1796.62</v>
+        <v>1230.0</v>
       </c>
       <c r="M15" t="n" s="0">
-        <v>1256.11</v>
+        <v>1523.25</v>
       </c>
       <c r="N15" t="n" s="0">
-        <v>1551.69</v>
+        <v>1914.54</v>
       </c>
       <c r="O15" t="n" s="0">
-        <v>1919.21</v>
+        <v>1965.69</v>
       </c>
     </row>
     <row r="16">
@@ -970,40 +970,40 @@
         <v>44</v>
       </c>
       <c r="D16" t="n" s="0">
-        <v>1572.4</v>
+        <v>1273.85</v>
       </c>
       <c r="E16" t="n" s="0">
-        <v>1662.24</v>
+        <v>1769.94</v>
       </c>
       <c r="F16" t="n" s="0">
-        <v>1469.57</v>
+        <v>1552.68</v>
       </c>
       <c r="G16" t="n" s="0">
-        <v>1480.1</v>
+        <v>1539.03</v>
       </c>
       <c r="H16" t="n" s="0">
-        <v>1449.35</v>
+        <v>1507.69</v>
       </c>
       <c r="I16" t="n" s="0">
-        <v>1347.06</v>
+        <v>1931.74</v>
       </c>
       <c r="J16" t="n" s="0">
-        <v>1609.02</v>
+        <v>1502.11</v>
       </c>
       <c r="K16" t="n" s="0">
-        <v>1273.22</v>
+        <v>1830.88</v>
       </c>
       <c r="L16" t="n" s="0">
-        <v>1999.21</v>
+        <v>1468.41</v>
       </c>
       <c r="M16" t="n" s="0">
-        <v>1652.65</v>
+        <v>1520.13</v>
       </c>
       <c r="N16" t="n" s="0">
-        <v>1242.36</v>
+        <v>1907.54</v>
       </c>
       <c r="O16" t="n" s="0">
-        <v>1419.46</v>
+        <v>1554.04</v>
       </c>
     </row>
     <row r="17">
@@ -1017,40 +1017,40 @@
         <v>46</v>
       </c>
       <c r="D17" t="n" s="0">
-        <v>1644.72</v>
+        <v>1954.97</v>
       </c>
       <c r="E17" t="n" s="0">
-        <v>1229.97</v>
+        <v>1225.25</v>
       </c>
       <c r="F17" t="n" s="0">
-        <v>1488.7</v>
+        <v>1255.79</v>
       </c>
       <c r="G17" t="n" s="0">
-        <v>1686.27</v>
+        <v>1530.95</v>
       </c>
       <c r="H17" t="n" s="0">
-        <v>1756.83</v>
+        <v>1540.82</v>
       </c>
       <c r="I17" t="n" s="0">
-        <v>1301.32</v>
+        <v>1889.87</v>
       </c>
       <c r="J17" t="n" s="0">
-        <v>1343.37</v>
+        <v>1385.57</v>
       </c>
       <c r="K17" t="n" s="0">
-        <v>1387.11</v>
+        <v>1640.92</v>
       </c>
       <c r="L17" t="n" s="0">
-        <v>1293.65</v>
+        <v>1875.01</v>
       </c>
       <c r="M17" t="n" s="0">
-        <v>1543.75</v>
+        <v>1360.99</v>
       </c>
       <c r="N17" t="n" s="0">
-        <v>1424.9</v>
+        <v>1217.23</v>
       </c>
       <c r="O17" t="n" s="0">
-        <v>1470.82</v>
+        <v>1779.32</v>
       </c>
     </row>
     <row r="18">
@@ -1064,40 +1064,40 @@
         <v>48</v>
       </c>
       <c r="D18" t="n" s="0">
-        <v>1888.97</v>
+        <v>1585.17</v>
       </c>
       <c r="E18" t="n" s="0">
-        <v>1458.15</v>
+        <v>1558.2</v>
       </c>
       <c r="F18" t="n" s="0">
-        <v>1512.96</v>
+        <v>1269.42</v>
       </c>
       <c r="G18" t="n" s="0">
-        <v>1497.36</v>
+        <v>1586.87</v>
       </c>
       <c r="H18" t="n" s="0">
-        <v>1986.12</v>
+        <v>1458.61</v>
       </c>
       <c r="I18" t="n" s="0">
-        <v>1358.4</v>
+        <v>1542.43</v>
       </c>
       <c r="J18" t="n" s="0">
-        <v>1652.01</v>
+        <v>1504.88</v>
       </c>
       <c r="K18" t="n" s="0">
-        <v>1978.55</v>
+        <v>1664.36</v>
       </c>
       <c r="L18" t="n" s="0">
-        <v>1326.51</v>
+        <v>1866.31</v>
       </c>
       <c r="M18" t="n" s="0">
-        <v>1609.6</v>
+        <v>1838.09</v>
       </c>
       <c r="N18" t="n" s="0">
-        <v>1720.53</v>
+        <v>1748.64</v>
       </c>
       <c r="O18" t="n" s="0">
-        <v>1969.18</v>
+        <v>1770.15</v>
       </c>
     </row>
     <row r="19">
@@ -1111,40 +1111,40 @@
         <v>50</v>
       </c>
       <c r="D19" t="n" s="0">
-        <v>1640.25</v>
+        <v>1507.79</v>
       </c>
       <c r="E19" t="n" s="0">
-        <v>1263.74</v>
+        <v>1556.48</v>
       </c>
       <c r="F19" t="n" s="0">
-        <v>1717.2</v>
+        <v>1247.49</v>
       </c>
       <c r="G19" t="n" s="0">
-        <v>1226.4</v>
+        <v>1904.57</v>
       </c>
       <c r="H19" t="n" s="0">
-        <v>1349.62</v>
+        <v>1292.97</v>
       </c>
       <c r="I19" t="n" s="0">
-        <v>1785.9</v>
+        <v>1787.56</v>
       </c>
       <c r="J19" t="n" s="0">
-        <v>1790.43</v>
+        <v>1890.68</v>
       </c>
       <c r="K19" t="n" s="0">
-        <v>1311.73</v>
+        <v>1817.87</v>
       </c>
       <c r="L19" t="n" s="0">
-        <v>1484.45</v>
+        <v>1740.68</v>
       </c>
       <c r="M19" t="n" s="0">
-        <v>1733.46</v>
+        <v>1871.87</v>
       </c>
       <c r="N19" t="n" s="0">
-        <v>1639.16</v>
+        <v>1787.08</v>
       </c>
       <c r="O19" t="n" s="0">
-        <v>1892.52</v>
+        <v>1734.77</v>
       </c>
     </row>
     <row r="20">
@@ -1158,40 +1158,40 @@
         <v>52</v>
       </c>
       <c r="D20" t="n" s="0">
-        <v>1221.8</v>
+        <v>1461.43</v>
       </c>
       <c r="E20" t="n" s="0">
-        <v>1645.32</v>
+        <v>1533.79</v>
       </c>
       <c r="F20" t="n" s="0">
-        <v>1738.02</v>
+        <v>1495.48</v>
       </c>
       <c r="G20" t="n" s="0">
-        <v>1606.52</v>
+        <v>1571.32</v>
       </c>
       <c r="H20" t="n" s="0">
-        <v>1300.4</v>
+        <v>1305.81</v>
       </c>
       <c r="I20" t="n" s="0">
-        <v>1817.85</v>
+        <v>1452.14</v>
       </c>
       <c r="J20" t="n" s="0">
-        <v>1891.09</v>
+        <v>1429.72</v>
       </c>
       <c r="K20" t="n" s="0">
-        <v>1985.3</v>
+        <v>1626.32</v>
       </c>
       <c r="L20" t="n" s="0">
-        <v>1623.95</v>
+        <v>1597.51</v>
       </c>
       <c r="M20" t="n" s="0">
-        <v>1888.54</v>
+        <v>1263.21</v>
       </c>
       <c r="N20" t="n" s="0">
-        <v>1494.14</v>
+        <v>1811.9</v>
       </c>
       <c r="O20" t="n" s="0">
-        <v>1289.19</v>
+        <v>1461.86</v>
       </c>
     </row>
     <row r="21">
@@ -1205,40 +1205,40 @@
         <v>54</v>
       </c>
       <c r="D21" t="n" s="0">
-        <v>1255.21</v>
+        <v>1333.96</v>
       </c>
       <c r="E21" t="n" s="0">
-        <v>1818.13</v>
+        <v>1636.27</v>
       </c>
       <c r="F21" t="n" s="0">
-        <v>1786.08</v>
+        <v>1222.08</v>
       </c>
       <c r="G21" t="n" s="0">
-        <v>1488.69</v>
+        <v>1844.48</v>
       </c>
       <c r="H21" t="n" s="0">
-        <v>1516.61</v>
+        <v>1925.25</v>
       </c>
       <c r="I21" t="n" s="0">
-        <v>1356.3</v>
+        <v>1930.88</v>
       </c>
       <c r="J21" t="n" s="0">
-        <v>1295.95</v>
+        <v>1493.97</v>
       </c>
       <c r="K21" t="n" s="0">
-        <v>1634.03</v>
+        <v>1200.5</v>
       </c>
       <c r="L21" t="n" s="0">
-        <v>1650.82</v>
+        <v>1555.68</v>
       </c>
       <c r="M21" t="n" s="0">
-        <v>1795.66</v>
+        <v>1439.96</v>
       </c>
       <c r="N21" t="n" s="0">
-        <v>1642.98</v>
+        <v>1431.96</v>
       </c>
       <c r="O21" t="n" s="0">
-        <v>1686.78</v>
+        <v>1446.04</v>
       </c>
     </row>
     <row r="22">
@@ -1252,40 +1252,40 @@
         <v>56</v>
       </c>
       <c r="D22" t="n" s="0">
-        <v>1458.53</v>
+        <v>1990.36</v>
       </c>
       <c r="E22" t="n" s="0">
-        <v>1763.38</v>
+        <v>1942.09</v>
       </c>
       <c r="F22" t="n" s="0">
-        <v>1822.39</v>
+        <v>1975.21</v>
       </c>
       <c r="G22" t="n" s="0">
-        <v>1344.47</v>
+        <v>1484.39</v>
       </c>
       <c r="H22" t="n" s="0">
-        <v>1718.7</v>
+        <v>1612.63</v>
       </c>
       <c r="I22" t="n" s="0">
-        <v>1569.03</v>
+        <v>1830.92</v>
       </c>
       <c r="J22" t="n" s="0">
-        <v>1511.02</v>
+        <v>1410.91</v>
       </c>
       <c r="K22" t="n" s="0">
-        <v>1270.93</v>
+        <v>1720.37</v>
       </c>
       <c r="L22" t="n" s="0">
-        <v>1809.63</v>
+        <v>1466.44</v>
       </c>
       <c r="M22" t="n" s="0">
-        <v>1822.16</v>
+        <v>1859.47</v>
       </c>
       <c r="N22" t="n" s="0">
-        <v>1752.33</v>
+        <v>1439.03</v>
       </c>
       <c r="O22" t="n" s="0">
-        <v>1852.59</v>
+        <v>1623.25</v>
       </c>
     </row>
     <row r="23">
@@ -1299,40 +1299,40 @@
         <v>58</v>
       </c>
       <c r="D23" t="n" s="0">
-        <v>1988.14</v>
+        <v>1890.81</v>
       </c>
       <c r="E23" t="n" s="0">
-        <v>1652.26</v>
+        <v>1531.03</v>
       </c>
       <c r="F23" t="n" s="0">
-        <v>1431.03</v>
+        <v>1317.02</v>
       </c>
       <c r="G23" t="n" s="0">
-        <v>1532.42</v>
+        <v>1477.04</v>
       </c>
       <c r="H23" t="n" s="0">
-        <v>1246.52</v>
+        <v>1572.27</v>
       </c>
       <c r="I23" t="n" s="0">
-        <v>1908.69</v>
+        <v>1388.6</v>
       </c>
       <c r="J23" t="n" s="0">
-        <v>1823.6</v>
+        <v>1563.51</v>
       </c>
       <c r="K23" t="n" s="0">
-        <v>1330.76</v>
+        <v>1388.85</v>
       </c>
       <c r="L23" t="n" s="0">
-        <v>1356.06</v>
+        <v>1303.86</v>
       </c>
       <c r="M23" t="n" s="0">
-        <v>1587.18</v>
+        <v>1498.71</v>
       </c>
       <c r="N23" t="n" s="0">
-        <v>1211.69</v>
+        <v>1976.06</v>
       </c>
       <c r="O23" t="n" s="0">
-        <v>1943.89</v>
+        <v>1383.01</v>
       </c>
     </row>
     <row r="24">
@@ -1346,40 +1346,40 @@
         <v>60</v>
       </c>
       <c r="D24" t="n" s="0">
-        <v>1218.68</v>
+        <v>1428.15</v>
       </c>
       <c r="E24" t="n" s="0">
-        <v>1424.66</v>
+        <v>1895.4</v>
       </c>
       <c r="F24" t="n" s="0">
-        <v>1470.91</v>
+        <v>1818.43</v>
       </c>
       <c r="G24" t="n" s="0">
-        <v>1218.59</v>
+        <v>1990.82</v>
       </c>
       <c r="H24" t="n" s="0">
-        <v>1786.61</v>
+        <v>1654.52</v>
       </c>
       <c r="I24" t="n" s="0">
-        <v>1923.11</v>
+        <v>1844.55</v>
       </c>
       <c r="J24" t="n" s="0">
-        <v>1898.77</v>
+        <v>1759.08</v>
       </c>
       <c r="K24" t="n" s="0">
-        <v>1232.6</v>
+        <v>1952.72</v>
       </c>
       <c r="L24" t="n" s="0">
-        <v>1373.52</v>
+        <v>1479.53</v>
       </c>
       <c r="M24" t="n" s="0">
-        <v>1608.1</v>
+        <v>1508.22</v>
       </c>
       <c r="N24" t="n" s="0">
-        <v>1520.86</v>
+        <v>1892.93</v>
       </c>
       <c r="O24" t="n" s="0">
-        <v>1268.29</v>
+        <v>1281.71</v>
       </c>
     </row>
     <row r="25">
@@ -1393,40 +1393,40 @@
         <v>62</v>
       </c>
       <c r="D25" t="n" s="0">
-        <v>1768.57</v>
+        <v>1202.42</v>
       </c>
       <c r="E25" t="n" s="0">
-        <v>1896.97</v>
+        <v>1533.25</v>
       </c>
       <c r="F25" t="n" s="0">
-        <v>1715.45</v>
+        <v>1554.6</v>
       </c>
       <c r="G25" t="n" s="0">
-        <v>1648.6</v>
+        <v>1593.97</v>
       </c>
       <c r="H25" t="n" s="0">
-        <v>1578.21</v>
+        <v>1515.95</v>
       </c>
       <c r="I25" t="n" s="0">
-        <v>1946.18</v>
+        <v>1257.95</v>
       </c>
       <c r="J25" t="n" s="0">
-        <v>1822.22</v>
+        <v>1831.77</v>
       </c>
       <c r="K25" t="n" s="0">
-        <v>1711.51</v>
+        <v>1694.53</v>
       </c>
       <c r="L25" t="n" s="0">
-        <v>1458.83</v>
+        <v>1866.26</v>
       </c>
       <c r="M25" t="n" s="0">
-        <v>1867.01</v>
+        <v>1825.11</v>
       </c>
       <c r="N25" t="n" s="0">
-        <v>1851.96</v>
+        <v>1913.46</v>
       </c>
       <c r="O25" t="n" s="0">
-        <v>1531.15</v>
+        <v>1312.94</v>
       </c>
     </row>
     <row r="26">
@@ -1440,40 +1440,40 @@
         <v>64</v>
       </c>
       <c r="D26" t="n" s="0">
-        <v>1566.71</v>
+        <v>1813.51</v>
       </c>
       <c r="E26" t="n" s="0">
-        <v>1743.11</v>
+        <v>1709.2</v>
       </c>
       <c r="F26" t="n" s="0">
-        <v>1289.43</v>
+        <v>1658.34</v>
       </c>
       <c r="G26" t="n" s="0">
-        <v>1750.96</v>
+        <v>1615.95</v>
       </c>
       <c r="H26" t="n" s="0">
-        <v>1839.89</v>
+        <v>1888.54</v>
       </c>
       <c r="I26" t="n" s="0">
-        <v>1353.16</v>
+        <v>1810.16</v>
       </c>
       <c r="J26" t="n" s="0">
-        <v>1682.64</v>
+        <v>1444.54</v>
       </c>
       <c r="K26" t="n" s="0">
-        <v>1476.14</v>
+        <v>1281.25</v>
       </c>
       <c r="L26" t="n" s="0">
-        <v>1439.89</v>
+        <v>1728.9</v>
       </c>
       <c r="M26" t="n" s="0">
-        <v>1796.27</v>
+        <v>1735.6</v>
       </c>
       <c r="N26" t="n" s="0">
-        <v>1637.67</v>
+        <v>1662.6</v>
       </c>
       <c r="O26" t="n" s="0">
-        <v>1379.65</v>
+        <v>1898.15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>